<commit_message>
Benchmark results - Lenovo - 30.05
</commit_message>
<xml_diff>
--- a/analysis/results/comparison.xlsx
+++ b/analysis/results/comparison.xlsx
@@ -561,16 +561,16 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.591</v>
+        <v>2.7345</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.5884</v>
+        <v>3.0025</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.6</v>
+        <v>2.1505</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.0338</v>
+        <v>0.099</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.8344</v>
+        <v>8.448499999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>1.7352</v>
+        <v>8.1427</v>
       </c>
       <c r="E3" t="n">
-        <v>1.8954</v>
+        <v>10.2463</v>
       </c>
       <c r="F3" t="n">
-        <v>0.039</v>
+        <v>0.1808</v>
       </c>
       <c r="G3" t="n">
         <v>291</v>
@@ -637,16 +637,16 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.8225</v>
+        <v>8.3546</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1.7324</v>
+        <v>8.116099999999999</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>2.0464</v>
+        <v>8.591699999999999</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.0397</v>
+        <v>0.1907</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>470</v>
@@ -679,19 +679,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.9837</v>
+        <v>9.0471</v>
       </c>
       <c r="D5" t="n">
-        <v>1.8822</v>
+        <v>8.841900000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>2.1022</v>
+        <v>9.446999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0706</v>
+        <v>0.3913</v>
       </c>
       <c r="G5" t="n">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -721,16 +721,16 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.1031</v>
+        <v>19.6907</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>3.9981</v>
+        <v>14.8089</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5.7935</v>
+        <v>23.1457</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.5306999999999999</v>
+        <v>2.5881</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>4608</v>
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>24.6815</v>
+        <v>83.73399999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>24.07</v>
+        <v>60.6766</v>
       </c>
       <c r="E7" t="n">
-        <v>27.0423</v>
+        <v>90.68089999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>6.4036</v>
+        <v>16.1958</v>
       </c>
       <c r="G7" t="n">
-        <v>41229</v>
+        <v>41230</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -805,19 +805,19 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>229.9332</v>
+        <v>581.9835</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>227.4311</v>
+        <v>557.9921000000001</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>233.7101</v>
+        <v>617.2495</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>63.8736</v>
+        <v>117.6768</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>407489</v>
+        <v>407490</v>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
@@ -847,16 +847,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.32250000000001</v>
+        <v>82.09739999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>78.64870000000001</v>
+        <v>81.7283</v>
       </c>
       <c r="E9" t="n">
-        <v>79.8386</v>
+        <v>83.33620000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>134.9707</v>
+        <v>133.6298</v>
       </c>
       <c r="G9" t="n">
         <v>291</v>
@@ -891,16 +891,16 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>79.0622</v>
+        <v>82.2367</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>78.6397</v>
+        <v>81.8796</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>79.6748</v>
+        <v>83.52809999999999</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>135.0102</v>
+        <v>133.6416</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>470</v>
@@ -933,19 +933,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.3746</v>
+        <v>82.6002</v>
       </c>
       <c r="D11" t="n">
-        <v>78.72110000000001</v>
+        <v>82.08069999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>79.90989999999999</v>
+        <v>83.6533</v>
       </c>
       <c r="F11" t="n">
-        <v>134.9749</v>
+        <v>133.8187</v>
       </c>
       <c r="G11" t="n">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -975,16 +975,16 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>79.56610000000001</v>
+        <v>83.6738</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>78.91719999999999</v>
+        <v>83.1567</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>80.5581</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>135.1111</v>
+        <v>135.6571</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>4608</v>
@@ -1017,19 +1017,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>82.62649999999999</v>
+        <v>93.5295</v>
       </c>
       <c r="D13" t="n">
-        <v>81.7621</v>
+        <v>92.2938</v>
       </c>
       <c r="E13" t="n">
-        <v>84.1232</v>
+        <v>95.24930000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>139.2621</v>
+        <v>151.2466</v>
       </c>
       <c r="G13" t="n">
-        <v>41229</v>
+        <v>41230</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -1059,19 +1059,19 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>110.7896</v>
+        <v>167.8835</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>109.3258</v>
+        <v>166.4792</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>115.1605</v>
+        <v>172.7899</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>178.3942</v>
+        <v>260.8272</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>407489</v>
+        <v>407490</v>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1215,13 +1215,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.591</v>
+        <v>2.7345</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5884</v>
+        <v>3.0025</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6</v>
+        <v>2.1505</v>
       </c>
       <c r="F2" t="n">
         <v>20</v>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>78.006</v>
+        <v>77.0438</v>
       </c>
       <c r="D3" t="n">
-        <v>78.0063</v>
+        <v>76.93600000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>77.5745</v>
+        <v>77.05419999999999</v>
       </c>
       <c r="F3" t="n">
         <v>20</v>
@@ -1339,13 +1339,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.8344</v>
+        <v>8.448499999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>1.7352</v>
+        <v>8.1427</v>
       </c>
       <c r="E4" t="n">
-        <v>1.8954</v>
+        <v>10.2463</v>
       </c>
       <c r="F4" t="n">
         <v>20</v>
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.8225</v>
+        <v>8.3546</v>
       </c>
       <c r="D5" t="n">
-        <v>1.7324</v>
+        <v>8.116099999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>2.0464</v>
+        <v>8.591699999999999</v>
       </c>
       <c r="F5" t="n">
         <v>20</v>
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.9837</v>
+        <v>9.0471</v>
       </c>
       <c r="D6" t="n">
-        <v>1.8822</v>
+        <v>8.841900000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>2.1022</v>
+        <v>9.446999999999999</v>
       </c>
       <c r="F6" t="n">
         <v>20</v>
@@ -1478,7 +1478,7 @@
         <v>65536</v>
       </c>
       <c r="H6" t="n">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1525,13 +1525,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4.1031</v>
+        <v>19.6907</v>
       </c>
       <c r="D7" t="n">
-        <v>3.9981</v>
+        <v>14.8089</v>
       </c>
       <c r="E7" t="n">
-        <v>5.7935</v>
+        <v>23.1457</v>
       </c>
       <c r="F7" t="n">
         <v>20</v>
@@ -1587,13 +1587,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24.6815</v>
+        <v>83.73399999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>24.07</v>
+        <v>60.6766</v>
       </c>
       <c r="E8" t="n">
-        <v>27.0423</v>
+        <v>90.68089999999999</v>
       </c>
       <c r="F8" t="n">
         <v>20</v>
@@ -1602,7 +1602,7 @@
         <v>10485760</v>
       </c>
       <c r="H8" t="n">
-        <v>41229</v>
+        <v>41230</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1649,13 +1649,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>229.9332</v>
+        <v>581.9835</v>
       </c>
       <c r="D9" t="n">
-        <v>227.4311</v>
+        <v>557.9921000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>233.7101</v>
+        <v>617.2495</v>
       </c>
       <c r="F9" t="n">
         <v>20</v>
@@ -1664,7 +1664,7 @@
         <v>104857600</v>
       </c>
       <c r="H9" t="n">
-        <v>407489</v>
+        <v>407490</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1711,13 +1711,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.32250000000001</v>
+        <v>82.09739999999999</v>
       </c>
       <c r="D10" t="n">
-        <v>78.64870000000001</v>
+        <v>81.7283</v>
       </c>
       <c r="E10" t="n">
-        <v>79.8386</v>
+        <v>83.33620000000001</v>
       </c>
       <c r="F10" t="n">
         <v>20</v>
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79.0622</v>
+        <v>82.2367</v>
       </c>
       <c r="D11" t="n">
-        <v>78.6397</v>
+        <v>81.8796</v>
       </c>
       <c r="E11" t="n">
-        <v>79.6748</v>
+        <v>83.52809999999999</v>
       </c>
       <c r="F11" t="n">
         <v>20</v>
@@ -1835,13 +1835,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>79.3746</v>
+        <v>82.6002</v>
       </c>
       <c r="D12" t="n">
-        <v>78.72110000000001</v>
+        <v>82.08069999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>79.90989999999999</v>
+        <v>83.6533</v>
       </c>
       <c r="F12" t="n">
         <v>20</v>
@@ -1897,13 +1897,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>79.56610000000001</v>
+        <v>83.6738</v>
       </c>
       <c r="D13" t="n">
-        <v>78.91719999999999</v>
+        <v>83.1567</v>
       </c>
       <c r="E13" t="n">
-        <v>80.5581</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="F13" t="n">
         <v>20</v>
@@ -1959,13 +1959,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>82.62649999999999</v>
+        <v>93.5295</v>
       </c>
       <c r="D14" t="n">
-        <v>81.7621</v>
+        <v>92.2938</v>
       </c>
       <c r="E14" t="n">
-        <v>84.1232</v>
+        <v>95.24930000000001</v>
       </c>
       <c r="F14" t="n">
         <v>20</v>
@@ -2021,13 +2021,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>110.7896</v>
+        <v>167.8835</v>
       </c>
       <c r="D15" t="n">
-        <v>109.3258</v>
+        <v>166.4792</v>
       </c>
       <c r="E15" t="n">
-        <v>115.1605</v>
+        <v>172.7899</v>
       </c>
       <c r="F15" t="n">
         <v>20</v>
@@ -2346,7 +2346,7 @@
         <v>10485760</v>
       </c>
       <c r="H20" t="n">
-        <v>41233</v>
+        <v>41232</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -2408,7 +2408,7 @@
         <v>104857600</v>
       </c>
       <c r="H21" t="n">
-        <v>407494</v>
+        <v>407495</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -2545,16 +2545,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.033797</v>
+        <v>0.099022</v>
       </c>
       <c r="D2" t="n">
-        <v>0.033797</v>
+        <v>0.099022</v>
       </c>
       <c r="E2" t="n">
-        <v>0.033797</v>
+        <v>0.099022</v>
       </c>
       <c r="F2" t="n">
-        <v>354219</v>
+        <v>118904</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -2595,16 +2595,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>78.080949</v>
+        <v>77.139971</v>
       </c>
       <c r="D3" t="n">
-        <v>78.080949</v>
+        <v>77.139971</v>
       </c>
       <c r="E3" t="n">
-        <v>78.080949</v>
+        <v>77.139971</v>
       </c>
       <c r="F3" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -2645,16 +2645,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.039048</v>
+        <v>0.180769</v>
       </c>
       <c r="D4" t="n">
-        <v>0.039048</v>
+        <v>0.180769</v>
       </c>
       <c r="E4" t="n">
-        <v>0.039048</v>
+        <v>0.180769</v>
       </c>
       <c r="F4" t="n">
-        <v>306926</v>
+        <v>66375</v>
       </c>
       <c r="G4" t="n">
         <v>100</v>
@@ -2695,16 +2695,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.039704</v>
+        <v>0.190702</v>
       </c>
       <c r="D5" t="n">
-        <v>0.039704</v>
+        <v>0.190702</v>
       </c>
       <c r="E5" t="n">
-        <v>0.039704</v>
+        <v>0.190702</v>
       </c>
       <c r="F5" t="n">
-        <v>302426</v>
+        <v>60896</v>
       </c>
       <c r="G5" t="n">
         <v>1024</v>
@@ -2745,16 +2745,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.07062400000000001</v>
+        <v>0.391338</v>
       </c>
       <c r="D6" t="n">
-        <v>0.07062400000000001</v>
+        <v>0.391338</v>
       </c>
       <c r="E6" t="n">
-        <v>0.07062400000000001</v>
+        <v>0.391338</v>
       </c>
       <c r="F6" t="n">
-        <v>168949</v>
+        <v>30414</v>
       </c>
       <c r="G6" t="n">
         <v>65536</v>
@@ -2795,16 +2795,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.530674</v>
+        <v>2.58809</v>
       </c>
       <c r="D7" t="n">
-        <v>0.530674</v>
+        <v>2.58809</v>
       </c>
       <c r="E7" t="n">
-        <v>0.530674</v>
+        <v>2.58809</v>
       </c>
       <c r="F7" t="n">
-        <v>22809</v>
+        <v>4483</v>
       </c>
       <c r="G7" t="n">
         <v>1048576</v>
@@ -2845,16 +2845,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6.403598</v>
+        <v>16.195792</v>
       </c>
       <c r="D8" t="n">
-        <v>6.403598</v>
+        <v>16.195792</v>
       </c>
       <c r="E8" t="n">
-        <v>6.403598</v>
+        <v>16.195792</v>
       </c>
       <c r="F8" t="n">
-        <v>1839</v>
+        <v>692</v>
       </c>
       <c r="G8" t="n">
         <v>10485760</v>
@@ -2895,16 +2895,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>63.873602</v>
+        <v>117.6768</v>
       </c>
       <c r="D9" t="n">
-        <v>63.873602</v>
+        <v>117.6768</v>
       </c>
       <c r="E9" t="n">
-        <v>63.873602</v>
+        <v>117.6768</v>
       </c>
       <c r="F9" t="n">
-        <v>186</v>
+        <v>99</v>
       </c>
       <c r="G9" t="n">
         <v>104857600</v>
@@ -2945,16 +2945,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>134.970682</v>
+        <v>133.629756</v>
       </c>
       <c r="D10" t="n">
-        <v>134.970682</v>
+        <v>133.629756</v>
       </c>
       <c r="E10" t="n">
-        <v>134.970682</v>
+        <v>133.629756</v>
       </c>
       <c r="F10" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G10" t="n">
         <v>100</v>
@@ -2995,13 +2995,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>135.010171</v>
+        <v>133.641558</v>
       </c>
       <c r="D11" t="n">
-        <v>135.010171</v>
+        <v>133.641558</v>
       </c>
       <c r="E11" t="n">
-        <v>135.010171</v>
+        <v>133.641558</v>
       </c>
       <c r="F11" t="n">
         <v>88</v>
@@ -3045,16 +3045,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>134.974929</v>
+        <v>133.818745</v>
       </c>
       <c r="D12" t="n">
-        <v>134.974929</v>
+        <v>133.818745</v>
       </c>
       <c r="E12" t="n">
-        <v>134.974929</v>
+        <v>133.818745</v>
       </c>
       <c r="F12" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G12" t="n">
         <v>65536</v>
@@ -3095,13 +3095,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>135.11108</v>
+        <v>135.657121</v>
       </c>
       <c r="D13" t="n">
-        <v>135.11108</v>
+        <v>135.657121</v>
       </c>
       <c r="E13" t="n">
-        <v>135.11108</v>
+        <v>135.657121</v>
       </c>
       <c r="F13" t="n">
         <v>87</v>
@@ -3145,16 +3145,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>139.262086</v>
+        <v>151.246622</v>
       </c>
       <c r="D14" t="n">
-        <v>139.262086</v>
+        <v>151.246622</v>
       </c>
       <c r="E14" t="n">
-        <v>139.262086</v>
+        <v>151.246622</v>
       </c>
       <c r="F14" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="G14" t="n">
         <v>10485760</v>
@@ -3195,16 +3195,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>178.394207</v>
+        <v>260.827233</v>
       </c>
       <c r="D15" t="n">
-        <v>178.394207</v>
+        <v>260.827233</v>
       </c>
       <c r="E15" t="n">
-        <v>178.394207</v>
+        <v>260.827233</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="G15" t="n">
         <v>104857600</v>

</xml_diff>

<commit_message>
Benchmark results - Lenevo - 31.05
</commit_message>
<xml_diff>
--- a/analysis/results/comparison.xlsx
+++ b/analysis/results/comparison.xlsx
@@ -561,16 +561,16 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2.7345</v>
+        <v>2.7133</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>3.0025</v>
+        <v>2.7518</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.1505</v>
+        <v>1.9968</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.099</v>
+        <v>0.0978</v>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8.448499999999999</v>
+        <v>8.101900000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>8.1427</v>
+        <v>7.7829</v>
       </c>
       <c r="E3" t="n">
-        <v>10.2463</v>
+        <v>8.294</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1808</v>
+        <v>0.184</v>
       </c>
       <c r="G3" t="n">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="H3" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -637,21 +637,23 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>8.3546</v>
+        <v>8.189</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>8.116099999999999</v>
+        <v>8.016500000000001</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>8.591699999999999</v>
+        <v>8.8218</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1907</v>
+        <v>0.1873</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>470</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+        <v>1212</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>188</v>
+      </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="n">
@@ -679,21 +681,23 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9.0471</v>
+        <v>8.3102</v>
       </c>
       <c r="D5" t="n">
-        <v>8.841900000000001</v>
+        <v>7.9601</v>
       </c>
       <c r="E5" t="n">
-        <v>9.446999999999999</v>
+        <v>8.638199999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3913</v>
+        <v>0.3884</v>
       </c>
       <c r="G5" t="n">
-        <v>795</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
+        <v>65730</v>
+      </c>
+      <c r="H5" t="n">
+        <v>194</v>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
@@ -721,21 +725,23 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>19.6907</v>
+        <v>12.1119</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>14.8089</v>
+        <v>11.7958</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>23.1457</v>
+        <v>13.4565</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.5881</v>
+        <v>2.6814</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>4608</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+        <v>1048769</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>193</v>
+      </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="n">
@@ -763,21 +769,23 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>83.73399999999999</v>
+        <v>47.4337</v>
       </c>
       <c r="D7" t="n">
-        <v>60.6766</v>
+        <v>24.9077</v>
       </c>
       <c r="E7" t="n">
-        <v>90.68089999999999</v>
+        <v>52.66</v>
       </c>
       <c r="F7" t="n">
-        <v>16.1958</v>
+        <v>16.545</v>
       </c>
       <c r="G7" t="n">
-        <v>41230</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
+        <v>10485954</v>
+      </c>
+      <c r="H7" t="n">
+        <v>194</v>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
@@ -805,21 +813,23 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>581.9835</v>
+        <v>218.1371</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>557.9921000000001</v>
+        <v>205.2712</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>617.2495</v>
+        <v>231.876</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>117.6768</v>
+        <v>115.703</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>407490</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
+        <v>104857795</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>195</v>
+      </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="n">
@@ -847,22 +857,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>82.09739999999999</v>
+        <v>82.7146</v>
       </c>
       <c r="D9" t="n">
-        <v>81.7283</v>
+        <v>81.60850000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>83.33620000000001</v>
+        <v>83.4198</v>
       </c>
       <c r="F9" t="n">
-        <v>133.6298</v>
+        <v>133.6079</v>
       </c>
       <c r="G9" t="n">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="H9" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -891,21 +901,23 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>82.2367</v>
+        <v>82.9829</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>81.8796</v>
+        <v>81.8877</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>83.52809999999999</v>
+        <v>83.6682</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>133.6416</v>
+        <v>133.5487</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>470</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+        <v>1212</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>188</v>
+      </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="n">
@@ -933,21 +945,23 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>82.6002</v>
+        <v>82.2396</v>
       </c>
       <c r="D11" t="n">
-        <v>82.08069999999999</v>
+        <v>81.9419</v>
       </c>
       <c r="E11" t="n">
-        <v>83.6533</v>
+        <v>83.52030000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>133.8187</v>
+        <v>133.7631</v>
       </c>
       <c r="G11" t="n">
-        <v>795</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+        <v>65730</v>
+      </c>
+      <c r="H11" t="n">
+        <v>194</v>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
@@ -975,21 +989,23 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>83.6738</v>
+        <v>83.64</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>83.1567</v>
+        <v>82.96420000000001</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>84.79000000000001</v>
+        <v>84.6968</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>135.6571</v>
+        <v>135.5729</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>4608</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+        <v>1048769</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>193</v>
+      </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="n">
@@ -1017,21 +1033,23 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>93.5295</v>
+        <v>93.4248</v>
       </c>
       <c r="D13" t="n">
-        <v>92.2938</v>
+        <v>92.2539</v>
       </c>
       <c r="E13" t="n">
-        <v>95.24930000000001</v>
+        <v>95.3021</v>
       </c>
       <c r="F13" t="n">
-        <v>151.2466</v>
+        <v>151.261</v>
       </c>
       <c r="G13" t="n">
-        <v>41230</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>10485954</v>
+      </c>
+      <c r="H13" t="n">
+        <v>194</v>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
@@ -1059,21 +1077,23 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>167.8835</v>
+        <v>171.6824</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>166.4792</v>
+        <v>166.9473</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>172.7899</v>
+        <v>175.3099</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>260.8272</v>
+        <v>262.2133</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>407490</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+        <v>104857795</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>195</v>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="n">
@@ -1215,13 +1235,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.7345</v>
+        <v>2.7133</v>
       </c>
       <c r="D2" t="n">
-        <v>3.0025</v>
+        <v>2.7518</v>
       </c>
       <c r="E2" t="n">
-        <v>2.1505</v>
+        <v>1.9968</v>
       </c>
       <c r="F2" t="n">
         <v>20</v>
@@ -1277,13 +1297,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>77.0438</v>
+        <v>77.0132</v>
       </c>
       <c r="D3" t="n">
-        <v>76.93600000000001</v>
+        <v>76.96639999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>77.05419999999999</v>
+        <v>76.98609999999999</v>
       </c>
       <c r="F3" t="n">
         <v>20</v>
@@ -1339,13 +1359,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8.448499999999999</v>
+        <v>8.101900000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>8.1427</v>
+        <v>7.7829</v>
       </c>
       <c r="E4" t="n">
-        <v>10.2463</v>
+        <v>8.294</v>
       </c>
       <c r="F4" t="n">
         <v>20</v>
@@ -1354,10 +1374,10 @@
         <v>100</v>
       </c>
       <c r="H4" t="n">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="I4" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -1401,13 +1421,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8.3546</v>
+        <v>8.189</v>
       </c>
       <c r="D5" t="n">
-        <v>8.116099999999999</v>
+        <v>8.016500000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>8.591699999999999</v>
+        <v>8.8218</v>
       </c>
       <c r="F5" t="n">
         <v>20</v>
@@ -1416,10 +1436,10 @@
         <v>1024</v>
       </c>
       <c r="H5" t="n">
-        <v>470</v>
+        <v>1212</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>188</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -1463,13 +1483,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9.0471</v>
+        <v>8.3102</v>
       </c>
       <c r="D6" t="n">
-        <v>8.841900000000001</v>
+        <v>7.9601</v>
       </c>
       <c r="E6" t="n">
-        <v>9.446999999999999</v>
+        <v>8.638199999999999</v>
       </c>
       <c r="F6" t="n">
         <v>20</v>
@@ -1478,10 +1498,10 @@
         <v>65536</v>
       </c>
       <c r="H6" t="n">
-        <v>795</v>
+        <v>65730</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -1525,13 +1545,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.6907</v>
+        <v>12.1119</v>
       </c>
       <c r="D7" t="n">
-        <v>14.8089</v>
+        <v>11.7958</v>
       </c>
       <c r="E7" t="n">
-        <v>23.1457</v>
+        <v>13.4565</v>
       </c>
       <c r="F7" t="n">
         <v>20</v>
@@ -1540,10 +1560,10 @@
         <v>1048576</v>
       </c>
       <c r="H7" t="n">
-        <v>4608</v>
+        <v>1048769</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -1587,13 +1607,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>83.73399999999999</v>
+        <v>47.4337</v>
       </c>
       <c r="D8" t="n">
-        <v>60.6766</v>
+        <v>24.9077</v>
       </c>
       <c r="E8" t="n">
-        <v>90.68089999999999</v>
+        <v>52.66</v>
       </c>
       <c r="F8" t="n">
         <v>20</v>
@@ -1602,10 +1622,10 @@
         <v>10485760</v>
       </c>
       <c r="H8" t="n">
-        <v>41230</v>
+        <v>10485954</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -1649,13 +1669,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>581.9835</v>
+        <v>218.1371</v>
       </c>
       <c r="D9" t="n">
-        <v>557.9921000000001</v>
+        <v>205.2712</v>
       </c>
       <c r="E9" t="n">
-        <v>617.2495</v>
+        <v>231.876</v>
       </c>
       <c r="F9" t="n">
         <v>20</v>
@@ -1664,10 +1684,10 @@
         <v>104857600</v>
       </c>
       <c r="H9" t="n">
-        <v>407490</v>
+        <v>104857795</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>195</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1711,13 +1731,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>82.09739999999999</v>
+        <v>82.7146</v>
       </c>
       <c r="D10" t="n">
-        <v>81.7283</v>
+        <v>81.60850000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>83.33620000000001</v>
+        <v>83.4198</v>
       </c>
       <c r="F10" t="n">
         <v>20</v>
@@ -1773,13 +1793,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>82.2367</v>
+        <v>82.9829</v>
       </c>
       <c r="D11" t="n">
-        <v>81.8796</v>
+        <v>81.8877</v>
       </c>
       <c r="E11" t="n">
-        <v>83.52809999999999</v>
+        <v>83.6682</v>
       </c>
       <c r="F11" t="n">
         <v>20</v>
@@ -1835,13 +1855,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>82.6002</v>
+        <v>82.2396</v>
       </c>
       <c r="D12" t="n">
-        <v>82.08069999999999</v>
+        <v>81.9419</v>
       </c>
       <c r="E12" t="n">
-        <v>83.6533</v>
+        <v>83.52030000000001</v>
       </c>
       <c r="F12" t="n">
         <v>20</v>
@@ -1897,13 +1917,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>83.6738</v>
+        <v>83.64</v>
       </c>
       <c r="D13" t="n">
-        <v>83.1567</v>
+        <v>82.96420000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>84.79000000000001</v>
+        <v>84.6968</v>
       </c>
       <c r="F13" t="n">
         <v>20</v>
@@ -1959,13 +1979,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>93.5295</v>
+        <v>93.4248</v>
       </c>
       <c r="D14" t="n">
-        <v>92.2938</v>
+        <v>92.2539</v>
       </c>
       <c r="E14" t="n">
-        <v>95.24930000000001</v>
+        <v>95.3021</v>
       </c>
       <c r="F14" t="n">
         <v>20</v>
@@ -2021,13 +2041,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>167.8835</v>
+        <v>171.6824</v>
       </c>
       <c r="D15" t="n">
-        <v>166.4792</v>
+        <v>166.9473</v>
       </c>
       <c r="E15" t="n">
-        <v>172.7899</v>
+        <v>175.3099</v>
       </c>
       <c r="F15" t="n">
         <v>20</v>
@@ -2222,7 +2242,7 @@
         <v>65536</v>
       </c>
       <c r="H18" t="n">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -2346,7 +2366,7 @@
         <v>10485760</v>
       </c>
       <c r="H20" t="n">
-        <v>41232</v>
+        <v>41233</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -2408,7 +2428,7 @@
         <v>104857600</v>
       </c>
       <c r="H21" t="n">
-        <v>407495</v>
+        <v>407493</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -2545,16 +2565,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.099022</v>
+        <v>0.09780700000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.099022</v>
+        <v>0.09780700000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>0.099022</v>
+        <v>0.09780700000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>118904</v>
+        <v>118411</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -2595,13 +2615,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>77.139971</v>
+        <v>77.100269</v>
       </c>
       <c r="D3" t="n">
-        <v>77.139971</v>
+        <v>77.100269</v>
       </c>
       <c r="E3" t="n">
-        <v>77.139971</v>
+        <v>77.100269</v>
       </c>
       <c r="F3" t="n">
         <v>154</v>
@@ -2645,16 +2665,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.180769</v>
+        <v>0.184036</v>
       </c>
       <c r="D4" t="n">
-        <v>0.180769</v>
+        <v>0.184036</v>
       </c>
       <c r="E4" t="n">
-        <v>0.180769</v>
+        <v>0.184036</v>
       </c>
       <c r="F4" t="n">
-        <v>66375</v>
+        <v>61374</v>
       </c>
       <c r="G4" t="n">
         <v>100</v>
@@ -2695,16 +2715,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.190702</v>
+        <v>0.187327</v>
       </c>
       <c r="D5" t="n">
-        <v>0.190702</v>
+        <v>0.187327</v>
       </c>
       <c r="E5" t="n">
-        <v>0.190702</v>
+        <v>0.187327</v>
       </c>
       <c r="F5" t="n">
-        <v>60896</v>
+        <v>58887</v>
       </c>
       <c r="G5" t="n">
         <v>1024</v>
@@ -2745,16 +2765,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.391338</v>
+        <v>0.388424</v>
       </c>
       <c r="D6" t="n">
-        <v>0.391338</v>
+        <v>0.388424</v>
       </c>
       <c r="E6" t="n">
-        <v>0.391338</v>
+        <v>0.388424</v>
       </c>
       <c r="F6" t="n">
-        <v>30414</v>
+        <v>30134</v>
       </c>
       <c r="G6" t="n">
         <v>65536</v>
@@ -2795,16 +2815,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.58809</v>
+        <v>2.681385</v>
       </c>
       <c r="D7" t="n">
-        <v>2.58809</v>
+        <v>2.681385</v>
       </c>
       <c r="E7" t="n">
-        <v>2.58809</v>
+        <v>2.681385</v>
       </c>
       <c r="F7" t="n">
-        <v>4483</v>
+        <v>3849</v>
       </c>
       <c r="G7" t="n">
         <v>1048576</v>
@@ -2845,16 +2865,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>16.195792</v>
+        <v>16.545041</v>
       </c>
       <c r="D8" t="n">
-        <v>16.195792</v>
+        <v>16.545041</v>
       </c>
       <c r="E8" t="n">
-        <v>16.195792</v>
+        <v>16.545041</v>
       </c>
       <c r="F8" t="n">
-        <v>692</v>
+        <v>718</v>
       </c>
       <c r="G8" t="n">
         <v>10485760</v>
@@ -2895,16 +2915,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>117.6768</v>
+        <v>115.703007</v>
       </c>
       <c r="D9" t="n">
-        <v>117.6768</v>
+        <v>115.703007</v>
       </c>
       <c r="E9" t="n">
-        <v>117.6768</v>
+        <v>115.703007</v>
       </c>
       <c r="F9" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="G9" t="n">
         <v>104857600</v>
@@ -2945,13 +2965,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>133.629756</v>
+        <v>133.607901</v>
       </c>
       <c r="D10" t="n">
-        <v>133.629756</v>
+        <v>133.607901</v>
       </c>
       <c r="E10" t="n">
-        <v>133.629756</v>
+        <v>133.607901</v>
       </c>
       <c r="F10" t="n">
         <v>88</v>
@@ -2995,13 +3015,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>133.641558</v>
+        <v>133.548666</v>
       </c>
       <c r="D11" t="n">
-        <v>133.641558</v>
+        <v>133.548666</v>
       </c>
       <c r="E11" t="n">
-        <v>133.641558</v>
+        <v>133.548666</v>
       </c>
       <c r="F11" t="n">
         <v>88</v>
@@ -3045,13 +3065,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>133.818745</v>
+        <v>133.763144</v>
       </c>
       <c r="D12" t="n">
-        <v>133.818745</v>
+        <v>133.763144</v>
       </c>
       <c r="E12" t="n">
-        <v>133.818745</v>
+        <v>133.763144</v>
       </c>
       <c r="F12" t="n">
         <v>88</v>
@@ -3095,13 +3115,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>135.657121</v>
+        <v>135.572901</v>
       </c>
       <c r="D13" t="n">
-        <v>135.657121</v>
+        <v>135.572901</v>
       </c>
       <c r="E13" t="n">
-        <v>135.657121</v>
+        <v>135.572901</v>
       </c>
       <c r="F13" t="n">
         <v>87</v>
@@ -3145,13 +3165,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>151.246622</v>
+        <v>151.261037</v>
       </c>
       <c r="D14" t="n">
-        <v>151.246622</v>
+        <v>151.261037</v>
       </c>
       <c r="E14" t="n">
-        <v>151.246622</v>
+        <v>151.261037</v>
       </c>
       <c r="F14" t="n">
         <v>76</v>
@@ -3195,16 +3215,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>260.827233</v>
+        <v>262.213344</v>
       </c>
       <c r="D15" t="n">
-        <v>260.827233</v>
+        <v>262.213344</v>
       </c>
       <c r="E15" t="n">
-        <v>260.827233</v>
+        <v>262.213344</v>
       </c>
       <c r="F15" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G15" t="n">
         <v>104857600</v>

</xml_diff>